<commit_message>
Merge main into nr-doc-core-body-structure 2f3d0fbd2d393e3302be2936e179087cabac252b
</commit_message>
<xml_diff>
--- a/nr-doc-core-body-structure/ig/CodeSystem-fr-core-cs-method-collection.xlsx
+++ b/nr-doc-core-body-structure/ig/CodeSystem-fr-core-cs-method-collection.xlsx
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>FR Core CodeSystem Mode Validation Identite</t>
+    <t>FR Core CodeSystem Method Collection</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-28T09:03:50+00:00</t>
+    <t>2026-09-17T13:25:30+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>